<commit_message>
feat: unify HMI, robot, and simulation control paths
</commit_message>
<xml_diff>
--- a/docs/diagnostic_code_reference.xlsx
+++ b/docs/diagnostic_code_reference.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="진단·운용 코드" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'진단·운용 코드'!$A$1:$K$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'진단·운용 코드'!$A$1:$K$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11">
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14">
@@ -940,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:K141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6583,1327 +6583,1535 @@
       <c r="K111" s="15" t="inlineStr"/>
     </row>
     <row r="112">
-      <c r="A112" s="19" t="n">
-        <v>5105</v>
-      </c>
-      <c r="B112" s="20" t="inlineStr">
-        <is>
-          <t>BASE_CMD_CLAMPED</t>
-        </is>
-      </c>
-      <c r="C112" s="19" t="inlineStr">
-        <is>
-          <t>경고</t>
-        </is>
-      </c>
-      <c r="D112" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E112" s="21" t="inlineStr">
+      <c r="A112" s="15" t="n">
+        <v>5107</v>
+      </c>
+      <c r="B112" s="16" t="inlineStr">
+        <is>
+          <t>BASE_POSTURE_FAILED</t>
+        </is>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t>오류</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E112" s="17" t="inlineStr">
         <is>
           <t>본체</t>
         </is>
       </c>
-      <c r="F112" s="21" t="inlineStr">
-        <is>
-          <t>브릿지</t>
-        </is>
-      </c>
-      <c r="G112" s="22" t="inlineStr">
-        <is>
-          <t>조작 속도가 한도로 제한되었습니다</t>
-        </is>
-      </c>
-      <c r="H112" s="22" t="inlineStr">
-        <is>
-          <t>보낸 속도가 허용 한도를 넘어 한도값으로 줄여 실행했습니다.</t>
-        </is>
-      </c>
-      <c r="I112" s="22" t="inlineStr">
-        <is>
-          <t>조작 속도를 낮추십시오</t>
-        </is>
-      </c>
-      <c r="J112" s="20" t="inlineStr">
-        <is>
-          <t>cmd/cmd_vel</t>
-        </is>
-      </c>
-      <c r="K112" s="19" t="n">
-        <v>5</v>
-      </c>
+      <c r="F112" s="17" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="G112" s="18" t="inlineStr">
+        <is>
+          <t>자세 전환 실패</t>
+        </is>
+      </c>
+      <c r="H112" s="18" t="inlineStr">
+        <is>
+          <t>본체가 요청한 자세로 바꾸지 못했습니다. 지면 상태나 현재 자세 때문에 전환이 거부되었습니다.</t>
+        </is>
+      </c>
+      <c r="I112" s="18" t="inlineStr">
+        <is>
+          <t>로봇 주변에 걸리는 것이 없는지 확인하십시오
+평평한 바닥에서 다시 시도하십시오
+반복되면 담당자에게 알리십시오</t>
+        </is>
+      </c>
+      <c r="J112" s="16" t="inlineStr">
+        <is>
+          <t>cmd/base/posture</t>
+        </is>
+      </c>
+      <c r="K112" s="15" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="19" t="n">
+        <v>5105</v>
+      </c>
+      <c r="B113" s="20" t="inlineStr">
+        <is>
+          <t>BASE_CMD_CLAMPED</t>
+        </is>
+      </c>
+      <c r="C113" s="19" t="inlineStr">
+        <is>
+          <t>경고</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E113" s="21" t="inlineStr">
+        <is>
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F113" s="21" t="inlineStr">
+        <is>
+          <t>브릿지</t>
+        </is>
+      </c>
+      <c r="G113" s="22" t="inlineStr">
+        <is>
+          <t>조작 속도가 한도로 제한되었습니다</t>
+        </is>
+      </c>
+      <c r="H113" s="22" t="inlineStr">
+        <is>
+          <t>보낸 속도가 허용 한도를 넘어 한도값으로 줄여 실행했습니다.</t>
+        </is>
+      </c>
+      <c r="I113" s="22" t="inlineStr">
+        <is>
+          <t>조작 속도를 낮추십시오</t>
+        </is>
+      </c>
+      <c r="J113" s="20" t="inlineStr">
+        <is>
+          <t>cmd/cmd_vel</t>
+        </is>
+      </c>
+      <c r="K113" s="19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="19" t="n">
         <v>5106</v>
       </c>
-      <c r="B113" s="20" t="inlineStr">
+      <c r="B114" s="20" t="inlineStr">
         <is>
           <t>BASE_ODOM_STALE</t>
         </is>
       </c>
-      <c r="C113" s="19" t="inlineStr">
+      <c r="C114" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D113" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E113" s="21" t="inlineStr">
+      <c r="D114" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E114" s="21" t="inlineStr">
         <is>
           <t>본체</t>
         </is>
       </c>
-      <c r="F113" s="21" t="inlineStr">
+      <c r="F114" s="21" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G113" s="22" t="inlineStr">
+      <c r="G114" s="22" t="inlineStr">
         <is>
           <t>주행 거리 정보가 오래되었습니다</t>
         </is>
       </c>
-      <c r="H113" s="22" t="inlineStr">
+      <c r="H114" s="22" t="inlineStr">
         <is>
           <t>본체에서 이동 정보가 갱신되지 않습니다. 정지 여부를 판단할 수 없어 촬영이 거부됩니다.</t>
         </is>
       </c>
-      <c r="I113" s="22" t="inlineStr">
+      <c r="I114" s="22" t="inlineStr">
         <is>
           <t>본체 연결을 확인하십시오
 증상이 이어지면 로봇을 재시작하십시오</t>
         </is>
       </c>
-      <c r="J113" s="20" t="inlineStr">
+      <c r="J114" s="20" t="inlineStr">
         <is>
           <t>state/pose</t>
         </is>
       </c>
-      <c r="K113" s="19" t="n">
+      <c r="K114" s="19" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="11" t="n">
+    <row r="115">
+      <c r="A115" s="19" t="n">
+        <v>5108</v>
+      </c>
+      <c r="B115" s="20" t="inlineStr">
+        <is>
+          <t>BASE_POSTURE_BLOCKED</t>
+        </is>
+      </c>
+      <c r="C115" s="19" t="inlineStr">
+        <is>
+          <t>경고</t>
+        </is>
+      </c>
+      <c r="D115" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E115" s="21" t="inlineStr">
+        <is>
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F115" s="21" t="inlineStr">
+        <is>
+          <t>브릿지</t>
+        </is>
+      </c>
+      <c r="G115" s="22" t="inlineStr">
+        <is>
+          <t>자세 전환 거부 — 선행 조건 미충족</t>
+        </is>
+      </c>
+      <c r="H115" s="22" t="inlineStr">
+        <is>
+          <t>로봇팔이 동작 중이거나 본체가 이동 중이라 자세를 바꾸지 않았습니다. 팔이 펴진 채 앉으면 차체나 바닥에 부딪힙니다.</t>
+        </is>
+      </c>
+      <c r="I115" s="22" t="inlineStr">
+        <is>
+          <t>로봇팔을 정지시키고 접은 뒤 다시 시도하십시오
+본체가 완전히 멈춘 것을 확인하십시오</t>
+        </is>
+      </c>
+      <c r="J115" s="20" t="inlineStr">
+        <is>
+          <t>cmd/base/posture</t>
+        </is>
+      </c>
+      <c r="K115" s="19" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="19" t="n">
+        <v>5110</v>
+      </c>
+      <c r="B116" s="20" t="inlineStr">
+        <is>
+          <t>BASE_POSTURE_SIMULATED</t>
+        </is>
+      </c>
+      <c r="C116" s="19" t="inlineStr">
+        <is>
+          <t>경고</t>
+        </is>
+      </c>
+      <c r="D116" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E116" s="21" t="inlineStr">
+        <is>
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F116" s="21" t="inlineStr">
+        <is>
+          <t>브릿지</t>
+        </is>
+      </c>
+      <c r="G116" s="22" t="inlineStr">
+        <is>
+          <t>자세 전환을 모의로 처리했습니다</t>
+        </is>
+      </c>
+      <c r="H116" s="22" t="inlineStr">
+        <is>
+          <t>본체 드라이버가 없는 상태에서 base.posture_dry_run 이 켜져 있어, 로봇은 움직이지 않고 상태만 바뀌었습니다. 시뮬레이터 설정입니다.</t>
+        </is>
+      </c>
+      <c r="I116" s="22" t="inlineStr">
+        <is>
+          <t>실기에서 이 알람이 보이면 base.posture_dry_run 을 끄십시오
+본체 드라이버가 올라와 있는지 확인하십시오</t>
+        </is>
+      </c>
+      <c r="J116" s="20" t="inlineStr">
+        <is>
+          <t>state/base</t>
+        </is>
+      </c>
+      <c r="K116" s="19" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="27" t="n">
+        <v>5109</v>
+      </c>
+      <c r="B117" s="28" t="inlineStr">
+        <is>
+          <t>BASE_POSTURE_CHANGED</t>
+        </is>
+      </c>
+      <c r="C117" s="27" t="inlineStr">
+        <is>
+          <t>정상</t>
+        </is>
+      </c>
+      <c r="D117" s="27" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E117" s="29" t="inlineStr">
+        <is>
+          <t>본체</t>
+        </is>
+      </c>
+      <c r="F117" s="29" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="G117" s="30" t="inlineStr">
+        <is>
+          <t>자세 전환 완료</t>
+        </is>
+      </c>
+      <c r="H117" s="30" t="inlineStr">
+        <is>
+          <t>본체가 요청한 자세로 바뀌었습니다.</t>
+        </is>
+      </c>
+      <c r="I117" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J117" s="28" t="inlineStr">
+        <is>
+          <t>state/base</t>
+        </is>
+      </c>
+      <c r="K117" s="27" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="n">
         <v>6001</v>
       </c>
-      <c r="B114" s="12" t="inlineStr">
+      <c r="B118" s="12" t="inlineStr">
         <is>
           <t>CAPTURE_SPOOL_FULL</t>
         </is>
       </c>
-      <c r="C114" s="11" t="inlineStr">
+      <c r="C118" s="11" t="inlineStr">
         <is>
           <t>치명</t>
         </is>
       </c>
-      <c r="D114" s="11" t="inlineStr">
+      <c r="D118" s="11" t="inlineStr">
         <is>
           <t>유지</t>
         </is>
       </c>
-      <c r="E114" s="13" t="inlineStr">
+      <c r="E118" s="13" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F114" s="13" t="inlineStr">
+      <c r="F118" s="13" t="inlineStr">
         <is>
           <t>저장소</t>
         </is>
       </c>
-      <c r="G114" s="14" t="inlineStr">
+      <c r="G118" s="14" t="inlineStr">
         <is>
           <t>로봇 저장 공간 부족 — 촬영 중단</t>
         </is>
       </c>
-      <c r="H114" s="14" t="inlineStr">
+      <c r="H118" s="14" t="inlineStr">
         <is>
           <t>로봇 안의 저장 공간이 거의 찼습니다. 저장 장치로 전송이 밀렸을 가능성이 높습니다.</t>
         </is>
       </c>
-      <c r="I114" s="14" t="inlineStr">
+      <c r="I118" s="14" t="inlineStr">
         <is>
           <t>저장 장치 연결 상태를 확인하십시오
 전송이 재개되면 자동으로 해소됩니다
 기존 촬영 데이터를 덮어쓰지 않습니다 — 공간이 확보될 때까지 촬영이 멈춥니다</t>
         </is>
       </c>
-      <c r="J114" s="12" t="inlineStr">
+      <c r="J118" s="12" t="inlineStr">
         <is>
           <t>state/capture_spool</t>
         </is>
       </c>
-      <c r="K114" s="11" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="15" t="n">
+      <c r="K118" s="11" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="15" t="n">
         <v>6002</v>
       </c>
-      <c r="B115" s="16" t="inlineStr">
+      <c r="B119" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_ENCODE_FAIL</t>
         </is>
       </c>
-      <c r="C115" s="15" t="inlineStr">
+      <c r="C119" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E115" s="17" t="inlineStr">
+      <c r="D119" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E119" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F115" s="17" t="inlineStr">
+      <c r="F119" s="17" t="inlineStr">
         <is>
           <t>브릿지</t>
         </is>
       </c>
-      <c r="G115" s="18" t="inlineStr">
+      <c r="G119" s="18" t="inlineStr">
         <is>
           <t>사진을 만들지 못했습니다</t>
         </is>
       </c>
-      <c r="H115" s="18" t="inlineStr">
+      <c r="H119" s="18" t="inlineStr">
         <is>
           <t>카메라 영상 형식을 사진으로 바꾸지 못했습니다.</t>
         </is>
       </c>
-      <c r="I115" s="18" t="inlineStr">
+      <c r="I119" s="18" t="inlineStr">
         <is>
           <t>담당자에게 알리십시오 — 카메라 설정을 확인해야 합니다</t>
         </is>
       </c>
-      <c r="J115" s="16" t="inlineStr">
+      <c r="J119" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K115" s="15" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="15" t="n">
+      <c r="K119" s="15" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="15" t="n">
         <v>6003</v>
       </c>
-      <c r="B116" s="16" t="inlineStr">
+      <c r="B120" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_ESTOP_BLOCKED</t>
         </is>
       </c>
-      <c r="C116" s="15" t="inlineStr">
+      <c r="C120" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E116" s="17" t="inlineStr">
+      <c r="D120" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F116" s="17" t="inlineStr">
+      <c r="F120" s="17" t="inlineStr">
         <is>
           <t>브릿지</t>
         </is>
       </c>
-      <c r="G116" s="18" t="inlineStr">
+      <c r="G120" s="18" t="inlineStr">
         <is>
           <t>E-Stop 중에는 촬영하지 않습니다</t>
         </is>
       </c>
-      <c r="H116" s="18" t="inlineStr">
+      <c r="H120" s="18" t="inlineStr">
         <is>
           <t>비상정지 상태에서는 촬영을 실행하지 않습니다.</t>
         </is>
       </c>
-      <c r="I116" s="18" t="inlineStr">
+      <c r="I120" s="18" t="inlineStr">
         <is>
           <t>E-Stop 을 해제한 뒤 다시 시도하십시오</t>
         </is>
       </c>
-      <c r="J116" s="16" t="inlineStr">
+      <c r="J120" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K116" s="15" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="15" t="n">
+      <c r="K120" s="15" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="15" t="n">
         <v>6004</v>
       </c>
-      <c r="B117" s="16" t="inlineStr">
+      <c r="B121" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_FAIL</t>
         </is>
       </c>
-      <c r="C117" s="15" t="inlineStr">
+      <c r="C121" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D117" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E117" s="17" t="inlineStr">
+      <c r="D121" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E121" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F117" s="17" t="inlineStr">
+      <c r="F121" s="17" t="inlineStr">
         <is>
           <t>D455</t>
         </is>
       </c>
-      <c r="G117" s="18" t="inlineStr">
+      <c r="G121" s="18" t="inlineStr">
         <is>
           <t>촬영 실패</t>
         </is>
       </c>
-      <c r="H117" s="18" t="inlineStr">
+      <c r="H121" s="18" t="inlineStr">
         <is>
           <t>카메라가 응답하지 않거나 영상 취득에 실패했습니다.</t>
         </is>
       </c>
-      <c r="I117" s="18" t="inlineStr">
+      <c r="I121" s="18" t="inlineStr">
         <is>
           <t>카메라 연결과 전원을 확인하십시오
 수동 촬영 버튼으로 재시도하십시오</t>
         </is>
       </c>
-      <c r="J117" s="16" t="inlineStr">
+      <c r="J121" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K117" s="15" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="15" t="n">
+      <c r="K121" s="15" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="15" t="n">
         <v>6005</v>
       </c>
-      <c r="B118" s="16" t="inlineStr">
+      <c r="B122" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_MOTION</t>
         </is>
       </c>
-      <c r="C118" s="15" t="inlineStr">
+      <c r="C122" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D118" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E118" s="17" t="inlineStr">
+      <c r="D122" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E122" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F118" s="17" t="inlineStr">
+      <c r="F122" s="17" t="inlineStr">
         <is>
           <t>브릿지</t>
         </is>
       </c>
-      <c r="G118" s="18" t="inlineStr">
+      <c r="G122" s="18" t="inlineStr">
         <is>
           <t>이동 중 촬영 시도 — 거부</t>
         </is>
       </c>
-      <c r="H118" s="18" t="inlineStr">
+      <c r="H122" s="18" t="inlineStr">
         <is>
           <t>로봇 또는 로봇팔이 정지하지 않은 상태에서 촬영이 요청되었습니다. 동적 촬영은 허용되지 않습니다.</t>
         </is>
       </c>
-      <c r="I118" s="18" t="inlineStr">
+      <c r="I122" s="18" t="inlineStr">
         <is>
           <t>정지 상태를 확인한 뒤 다시 촬영하십시오</t>
         </is>
       </c>
-      <c r="J118" s="16" t="inlineStr">
+      <c r="J122" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K118" s="15" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="15" t="n">
+      <c r="K122" s="15" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="15" t="n">
         <v>6006</v>
       </c>
-      <c r="B119" s="16" t="inlineStr">
+      <c r="B123" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_NAS_OFFLINE</t>
         </is>
       </c>
-      <c r="C119" s="15" t="inlineStr">
+      <c r="C123" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D119" s="15" t="inlineStr">
+      <c r="D123" s="15" t="inlineStr">
         <is>
           <t>짝 해제</t>
         </is>
       </c>
-      <c r="E119" s="17" t="inlineStr">
+      <c r="E123" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F119" s="17" t="inlineStr">
+      <c r="F123" s="17" t="inlineStr">
         <is>
           <t>NAS</t>
         </is>
       </c>
-      <c r="G119" s="18" t="inlineStr">
+      <c r="G123" s="18" t="inlineStr">
         <is>
           <t>저장 장치 연결 끊김 — 로봇에 임시 보관 중</t>
         </is>
       </c>
-      <c r="H119" s="18" t="inlineStr">
+      <c r="H123" s="18" t="inlineStr">
         <is>
           <t>촬영 데이터를 저장할 장치에 연결할 수 없습니다. 촬영은 계속되며 데이터는 로봇 안에 쌓입니다.</t>
         </is>
       </c>
-      <c r="I119" s="18" t="inlineStr">
+      <c r="I123" s="18" t="inlineStr">
         <is>
           <t>저장 장치 전원과 네트워크 연결을 확인하십시오
 로봇의 남은 저장 공간을 주시하십시오
 복구되면 밀린 파일이 자동으로 전송됩니다</t>
         </is>
       </c>
-      <c r="J119" s="16" t="inlineStr">
+      <c r="J123" s="16" t="inlineStr">
         <is>
           <t>state/capture_spool</t>
         </is>
       </c>
-      <c r="K119" s="15" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="15" t="n">
+      <c r="K123" s="15" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="15" t="n">
         <v>6007</v>
       </c>
-      <c r="B120" s="16" t="inlineStr">
+      <c r="B124" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_NAS_WRITE_FAIL</t>
         </is>
       </c>
-      <c r="C120" s="15" t="inlineStr">
+      <c r="C124" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D120" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E120" s="17" t="inlineStr">
+      <c r="D124" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E124" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F120" s="17" t="inlineStr">
+      <c r="F124" s="17" t="inlineStr">
         <is>
           <t>NAS</t>
         </is>
       </c>
-      <c r="G120" s="18" t="inlineStr">
+      <c r="G124" s="18" t="inlineStr">
         <is>
           <t>NAS 저장 실패</t>
         </is>
       </c>
-      <c r="H120" s="18" t="inlineStr">
+      <c r="H124" s="18" t="inlineStr">
         <is>
           <t>촬영 데이터를 내부망 NAS에 저장하지 못했습니다.</t>
         </is>
       </c>
-      <c r="I120" s="18" t="inlineStr">
+      <c r="I124" s="18" t="inlineStr">
         <is>
           <t>NAS 연결과 여유 용량을 확인하십시오
 데이터는 로봇 로컬에 임시 보관됩니다 — 복구 후 재전송하십시오</t>
         </is>
       </c>
-      <c r="J120" s="16" t="inlineStr"/>
-      <c r="K120" s="15" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="15" t="n">
+      <c r="J124" s="16" t="inlineStr"/>
+      <c r="K124" s="15" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="15" t="n">
         <v>6008</v>
       </c>
-      <c r="B121" s="16" t="inlineStr">
+      <c r="B125" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_NO_FRAME</t>
         </is>
       </c>
-      <c r="C121" s="15" t="inlineStr">
+      <c r="C125" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D121" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E121" s="17" t="inlineStr">
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E125" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F121" s="17" t="inlineStr">
+      <c r="F125" s="17" t="inlineStr">
         <is>
           <t>D455</t>
         </is>
       </c>
-      <c r="G121" s="18" t="inlineStr">
+      <c r="G125" s="18" t="inlineStr">
         <is>
           <t>카메라 영상이 없습니다</t>
         </is>
       </c>
-      <c r="H121" s="18" t="inlineStr">
+      <c r="H125" s="18" t="inlineStr">
         <is>
           <t>카메라에서 영상이 오지 않아 촬영할 수 없습니다.</t>
         </is>
       </c>
-      <c r="I121" s="18" t="inlineStr">
+      <c r="I125" s="18" t="inlineStr">
         <is>
           <t>카메라 케이블을 확인하십시오
 USB 를 뺐다가 다시 연결하십시오</t>
         </is>
       </c>
-      <c r="J121" s="16" t="inlineStr">
+      <c r="J125" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K121" s="15" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="15" t="n">
+      <c r="K125" s="15" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="15" t="n">
         <v>6009</v>
       </c>
-      <c r="B122" s="16" t="inlineStr">
+      <c r="B126" s="16" t="inlineStr">
         <is>
           <t>CAPTURE_SPOOL_MKDIR_FAIL</t>
         </is>
       </c>
-      <c r="C122" s="15" t="inlineStr">
+      <c r="C126" s="15" t="inlineStr">
         <is>
           <t>오류</t>
         </is>
       </c>
-      <c r="D122" s="15" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E122" s="17" t="inlineStr">
+      <c r="D126" s="15" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E126" s="17" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F122" s="17" t="inlineStr">
+      <c r="F126" s="17" t="inlineStr">
         <is>
           <t>저장소</t>
         </is>
       </c>
-      <c r="G122" s="18" t="inlineStr">
+      <c r="G126" s="18" t="inlineStr">
         <is>
           <t>저장 폴더를 만들지 못했습니다</t>
         </is>
       </c>
-      <c r="H122" s="18" t="inlineStr">
+      <c r="H126" s="18" t="inlineStr">
         <is>
           <t>촬영 파일을 둘 폴더를 만들지 못했습니다. 저장 공간이나 권한 문제입니다.</t>
         </is>
       </c>
-      <c r="I122" s="18" t="inlineStr">
+      <c r="I126" s="18" t="inlineStr">
         <is>
           <t>저장 공간을 확인하십시오
 담당자에게 알리십시오</t>
         </is>
       </c>
-      <c r="J122" s="16" t="inlineStr">
+      <c r="J126" s="16" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K122" s="15" t="inlineStr"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="19" t="n">
+      <c r="K126" s="15" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="19" t="n">
         <v>6010</v>
       </c>
-      <c r="B123" s="20" t="inlineStr">
+      <c r="B127" s="20" t="inlineStr">
         <is>
           <t>CAPTURE_DISABLED</t>
         </is>
       </c>
-      <c r="C123" s="19" t="inlineStr">
+      <c r="C127" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D123" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E123" s="21" t="inlineStr">
+      <c r="D127" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E127" s="21" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F123" s="21" t="inlineStr">
+      <c r="F127" s="21" t="inlineStr">
         <is>
           <t>브릿지</t>
         </is>
       </c>
-      <c r="G123" s="22" t="inlineStr">
+      <c r="G127" s="22" t="inlineStr">
         <is>
           <t>이 배포본에는 촬영 기능이 없습니다</t>
         </is>
       </c>
-      <c r="H123" s="22" t="inlineStr">
+      <c r="H127" s="22" t="inlineStr">
         <is>
           <t>현재 설치된 구성에 촬영 기능이 포함되어 있지 않습니다.</t>
         </is>
       </c>
-      <c r="I123" s="22" t="inlineStr">
+      <c r="I127" s="22" t="inlineStr">
         <is>
           <t>담당자에게 알리십시오</t>
         </is>
       </c>
-      <c r="J123" s="20" t="inlineStr">
+      <c r="J127" s="20" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K123" s="19" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="19" t="n">
+      <c r="K127" s="19" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="19" t="n">
         <v>6011</v>
       </c>
-      <c r="B124" s="20" t="inlineStr">
+      <c r="B128" s="20" t="inlineStr">
         <is>
           <t>CAPTURE_DISTANCE_UNKNOWN</t>
         </is>
       </c>
-      <c r="C124" s="19" t="inlineStr">
+      <c r="C128" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D124" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E124" s="21" t="inlineStr">
+      <c r="D128" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E128" s="21" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F124" s="21" t="inlineStr">
+      <c r="F128" s="21" t="inlineStr">
         <is>
           <t>D455</t>
         </is>
       </c>
-      <c r="G124" s="22" t="inlineStr">
+      <c r="G128" s="22" t="inlineStr">
         <is>
           <t>촬영거리를 측정하지 못했습니다</t>
         </is>
       </c>
-      <c r="H124" s="22" t="inlineStr">
+      <c r="H128" s="22" t="inlineStr">
         <is>
           <t>깊이 카메라가 거리를 재지 못했습니다. 사진은 저장되었으나 거리가 비어 있습니다.</t>
         </is>
       </c>
-      <c r="I124" s="22" t="inlineStr">
+      <c r="I128" s="22" t="inlineStr">
         <is>
           <t>대상과의 거리를 조정한 뒤 다시 촬영하십시오</t>
         </is>
       </c>
-      <c r="J124" s="20" t="inlineStr">
+      <c r="J128" s="20" t="inlineStr">
         <is>
           <t>capture/preview</t>
         </is>
       </c>
-      <c r="K124" s="19" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="19" t="n">
+      <c r="K128" s="19" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="19" t="n">
         <v>6012</v>
       </c>
-      <c r="B125" s="20" t="inlineStr">
+      <c r="B129" s="20" t="inlineStr">
         <is>
           <t>CAPTURE_METADATA_INCOMPLETE</t>
         </is>
       </c>
-      <c r="C125" s="19" t="inlineStr">
+      <c r="C129" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D125" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E125" s="21" t="inlineStr">
+      <c r="D129" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E129" s="21" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F125" s="21" t="inlineStr">
+      <c r="F129" s="21" t="inlineStr">
         <is>
           <t>브릿지</t>
         </is>
       </c>
-      <c r="G125" s="22" t="inlineStr">
+      <c r="G129" s="22" t="inlineStr">
         <is>
           <t>메타데이터 누락</t>
         </is>
       </c>
-      <c r="H125" s="22" t="inlineStr">
+      <c r="H129" s="22" t="inlineStr">
         <is>
           <t>차량번호·량번호·포인트ID 중 필수 항목이 비어 있습니다.</t>
         </is>
       </c>
-      <c r="I125" s="22" t="inlineStr">
+      <c r="I129" s="22" t="inlineStr">
         <is>
           <t>촬영 제어 패널에서 누락 항목을 입력하십시오
 누락 상태로 저장된 파일은 검수에서 제외될 수 있습니다</t>
         </is>
       </c>
-      <c r="J125" s="20" t="inlineStr"/>
-      <c r="K125" s="19" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="19" t="n">
+      <c r="J129" s="20" t="inlineStr"/>
+      <c r="K129" s="19" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="19" t="n">
         <v>6013</v>
       </c>
-      <c r="B126" s="20" t="inlineStr">
+      <c r="B130" s="20" t="inlineStr">
         <is>
           <t>CAPTURE_POSE_UNKNOWN</t>
         </is>
       </c>
-      <c r="C126" s="19" t="inlineStr">
+      <c r="C130" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D126" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E126" s="21" t="inlineStr">
+      <c r="D130" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E130" s="21" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F126" s="21" t="inlineStr">
+      <c r="F130" s="21" t="inlineStr">
         <is>
           <t>SLAM</t>
         </is>
       </c>
-      <c r="G126" s="22" t="inlineStr">
+      <c r="G130" s="22" t="inlineStr">
         <is>
           <t>촬영 위치를 기록하지 못했습니다</t>
         </is>
       </c>
-      <c r="H126" s="22" t="inlineStr">
+      <c r="H130" s="22" t="inlineStr">
         <is>
           <t>촬영 시각의 로봇 위치를 읽지 못했습니다. 사진은 저장되었으나 좌표가 비어 있습니다.</t>
         </is>
       </c>
-      <c r="I126" s="22" t="inlineStr">
+      <c r="I130" s="22" t="inlineStr">
         <is>
           <t>해당 사진의 위치 정보를 별도로 확인하십시오</t>
         </is>
       </c>
-      <c r="J126" s="20" t="inlineStr">
+      <c r="J130" s="20" t="inlineStr">
         <is>
           <t>capture/preview</t>
         </is>
       </c>
-      <c r="K126" s="19" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="19" t="n">
+      <c r="K130" s="19" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="19" t="n">
         <v>6014</v>
       </c>
-      <c r="B127" s="20" t="inlineStr">
+      <c r="B131" s="20" t="inlineStr">
         <is>
           <t>CAPTURE_UPLOAD_RETRY</t>
         </is>
       </c>
-      <c r="C127" s="19" t="inlineStr">
+      <c r="C131" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D127" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E127" s="21" t="inlineStr">
+      <c r="D131" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E131" s="21" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F127" s="21" t="inlineStr">
+      <c r="F131" s="21" t="inlineStr">
         <is>
           <t>NAS</t>
         </is>
       </c>
-      <c r="G127" s="22" t="inlineStr">
+      <c r="G131" s="22" t="inlineStr">
         <is>
           <t>촬영 데이터 전송 재시도</t>
         </is>
       </c>
-      <c r="H127" s="22" t="inlineStr">
+      <c r="H131" s="22" t="inlineStr">
         <is>
           <t>저장 장치로 보내다 실패해 다시 시도하고 있습니다. 무선 상태가 나쁠 때 흔합니다.</t>
         </is>
       </c>
-      <c r="I127" s="22" t="inlineStr">
+      <c r="I131" s="22" t="inlineStr">
         <is>
           <t>반복되면 무선 신호 세기와 저장 장치 상태를 확인하십시오</t>
         </is>
       </c>
-      <c r="J127" s="20" t="inlineStr">
+      <c r="J131" s="20" t="inlineStr">
         <is>
           <t>state/capture_spool</t>
         </is>
       </c>
-      <c r="K127" s="19" t="n">
+      <c r="K131" s="19" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="27" t="n">
+    <row r="132">
+      <c r="A132" s="27" t="n">
         <v>6015</v>
       </c>
-      <c r="B128" s="28" t="inlineStr">
+      <c r="B132" s="28" t="inlineStr">
         <is>
           <t>CAPTURE_OK</t>
         </is>
       </c>
-      <c r="C128" s="27" t="inlineStr">
+      <c r="C132" s="27" t="inlineStr">
         <is>
           <t>정상</t>
         </is>
       </c>
-      <c r="D128" s="27" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E128" s="29" t="inlineStr">
+      <c r="D132" s="27" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E132" s="29" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F128" s="29" t="inlineStr">
+      <c r="F132" s="29" t="inlineStr">
         <is>
           <t>D455</t>
         </is>
       </c>
-      <c r="G128" s="30" t="inlineStr">
+      <c r="G132" s="30" t="inlineStr">
         <is>
           <t>촬영 완료</t>
         </is>
       </c>
-      <c r="H128" s="30" t="inlineStr">
+      <c r="H132" s="30" t="inlineStr">
         <is>
           <t>정지 상태에서 촬영하고 메타데이터를 기록했습니다.</t>
         </is>
       </c>
-      <c r="I128" s="30" t="inlineStr">
+      <c r="I132" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J128" s="28" t="inlineStr">
+      <c r="J132" s="28" t="inlineStr">
         <is>
           <t>cmd/capture/trigger</t>
         </is>
       </c>
-      <c r="K128" s="27" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" s="27" t="n">
+      <c r="K132" s="27" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="27" t="n">
         <v>6016</v>
       </c>
-      <c r="B129" s="28" t="inlineStr">
+      <c r="B133" s="28" t="inlineStr">
         <is>
           <t>CAPTURE_UPLOAD_COMPLETE</t>
         </is>
       </c>
-      <c r="C129" s="27" t="inlineStr">
+      <c r="C133" s="27" t="inlineStr">
         <is>
           <t>정상</t>
         </is>
       </c>
-      <c r="D129" s="27" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E129" s="29" t="inlineStr">
+      <c r="D133" s="27" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E133" s="29" t="inlineStr">
         <is>
           <t>촬영</t>
         </is>
       </c>
-      <c r="F129" s="29" t="inlineStr">
+      <c r="F133" s="29" t="inlineStr">
         <is>
           <t>NAS</t>
         </is>
       </c>
-      <c r="G129" s="30" t="inlineStr">
+      <c r="G133" s="30" t="inlineStr">
         <is>
           <t>촬영 데이터 전송 완료</t>
         </is>
       </c>
-      <c r="H129" s="30" t="inlineStr">
+      <c r="H133" s="30" t="inlineStr">
         <is>
           <t>촬영한 사진이 모두 저장 장치로 옮겨지고 확인까지 끝났습니다.</t>
         </is>
       </c>
-      <c r="I129" s="30" t="inlineStr">
+      <c r="I133" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J129" s="28" t="inlineStr">
+      <c r="J133" s="28" t="inlineStr">
         <is>
           <t>state/capture_spool</t>
         </is>
       </c>
-      <c r="K129" s="27" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" s="11" t="n">
+      <c r="K133" s="27" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="n">
         <v>7001</v>
       </c>
-      <c r="B130" s="12" t="inlineStr">
+      <c r="B134" s="12" t="inlineStr">
         <is>
           <t>POWER_BATTERY_CRITICAL</t>
         </is>
       </c>
-      <c r="C130" s="11" t="inlineStr">
+      <c r="C134" s="11" t="inlineStr">
         <is>
           <t>치명</t>
         </is>
       </c>
-      <c r="D130" s="11" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E130" s="13" t="inlineStr">
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E134" s="13" t="inlineStr">
         <is>
           <t>전원</t>
         </is>
       </c>
-      <c r="F130" s="13" t="inlineStr">
+      <c r="F134" s="13" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G130" s="14" t="inlineStr">
+      <c r="G134" s="14" t="inlineStr">
         <is>
           <t>배터리 위험 수준</t>
         </is>
       </c>
-      <c r="H130" s="14" t="inlineStr">
+      <c r="H134" s="14" t="inlineStr">
         <is>
           <t>즉시 복귀가 필요한 수준입니다.</t>
         </is>
       </c>
-      <c r="I130" s="14" t="inlineStr">
+      <c r="I134" s="14" t="inlineStr">
         <is>
           <t>진행 중인 촬영을 중단하십시오
 충전 스테이션 복귀를 실행하십시오</t>
         </is>
       </c>
-      <c r="J130" s="12" t="inlineStr">
+      <c r="J134" s="12" t="inlineStr">
         <is>
           <t>state/battery</t>
         </is>
       </c>
-      <c r="K130" s="11" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" s="19" t="n">
+      <c r="K134" s="11" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="19" t="n">
         <v>7002</v>
       </c>
-      <c r="B131" s="20" t="inlineStr">
+      <c r="B135" s="20" t="inlineStr">
         <is>
           <t>POWER_BATTERY_LOW</t>
         </is>
       </c>
-      <c r="C131" s="19" t="inlineStr">
+      <c r="C135" s="19" t="inlineStr">
         <is>
           <t>경고</t>
         </is>
       </c>
-      <c r="D131" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E131" s="21" t="inlineStr">
+      <c r="D135" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E135" s="21" t="inlineStr">
         <is>
           <t>전원</t>
         </is>
       </c>
-      <c r="F131" s="21" t="inlineStr">
+      <c r="F135" s="21" t="inlineStr">
         <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G131" s="22" t="inlineStr">
+      <c r="G135" s="22" t="inlineStr">
         <is>
           <t>배터리 부족</t>
         </is>
       </c>
-      <c r="H131" s="22" t="inlineStr">
+      <c r="H135" s="22" t="inlineStr">
         <is>
           <t>배터리 잔량이 설정 임계 이하로 떨어졌습니다.</t>
         </is>
       </c>
-      <c r="I131" s="22" t="inlineStr">
+      <c r="I135" s="22" t="inlineStr">
         <is>
           <t>남은 점검 구간을 확인하십시오
 임계 이하에서는 충전 스테이션 복귀가 자동 실행됩니다</t>
         </is>
       </c>
-      <c r="J131" s="20" t="inlineStr">
+      <c r="J135" s="20" t="inlineStr">
         <is>
           <t>state/battery</t>
         </is>
       </c>
-      <c r="K131" s="19" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="23" t="n">
-        <v>7003</v>
-      </c>
-      <c r="B132" s="24" t="inlineStr">
-        <is>
-          <t>POWER_RETURN_TO_DOCK</t>
-        </is>
-      </c>
-      <c r="C132" s="23" t="inlineStr">
-        <is>
-          <t>정보</t>
-        </is>
-      </c>
-      <c r="D132" s="23" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E132" s="25" t="inlineStr">
-        <is>
-          <t>전원</t>
-        </is>
-      </c>
-      <c r="F132" s="25" t="inlineStr">
-        <is>
-          <t>미션 FSM</t>
-        </is>
-      </c>
-      <c r="G132" s="26" t="inlineStr">
-        <is>
-          <t>충전 스테이션 복귀</t>
-        </is>
-      </c>
-      <c r="H132" s="26" t="inlineStr">
-        <is>
-          <t>점검 완료 또는 배터리 부족으로 복귀 중입니다.</t>
-        </is>
-      </c>
-      <c r="I132" s="26" t="inlineStr">
-        <is>
-          <t>복귀 경로상 장애물이 없는지 확인하십시오</t>
-        </is>
-      </c>
-      <c r="J132" s="24" t="inlineStr">
-        <is>
-          <t>state/mission</t>
-        </is>
-      </c>
-      <c r="K132" s="23" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" s="27" t="n">
-        <v>7004</v>
-      </c>
-      <c r="B133" s="28" t="inlineStr">
-        <is>
-          <t>POWER_DOCKED</t>
-        </is>
-      </c>
-      <c r="C133" s="27" t="inlineStr">
-        <is>
-          <t>정상</t>
-        </is>
-      </c>
-      <c r="D133" s="27" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E133" s="29" t="inlineStr">
-        <is>
-          <t>전원</t>
-        </is>
-      </c>
-      <c r="F133" s="29" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="G133" s="30" t="inlineStr">
-        <is>
-          <t>충전 스테이션 도킹 완료</t>
-        </is>
-      </c>
-      <c r="H133" s="30" t="inlineStr">
-        <is>
-          <t>복귀와 충전 연결이 완료되었습니다.</t>
-        </is>
-      </c>
-      <c r="I133" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J133" s="28" t="inlineStr">
-        <is>
-          <t>state/mission</t>
-        </is>
-      </c>
-      <c r="K133" s="27" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="19" t="n">
-        <v>8001</v>
-      </c>
-      <c r="B134" s="20" t="inlineStr">
-        <is>
-          <t>AUDIT_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="C134" s="19" t="inlineStr">
-        <is>
-          <t>경고</t>
-        </is>
-      </c>
-      <c r="D134" s="19" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E134" s="21" t="inlineStr">
-        <is>
-          <t>조작 이력</t>
-        </is>
-      </c>
-      <c r="F134" s="21" t="inlineStr">
-        <is>
-          <t>관제</t>
-        </is>
-      </c>
-      <c r="G134" s="22" t="inlineStr">
-        <is>
-          <t>경고를 무시하고 강행</t>
-        </is>
-      </c>
-      <c r="H134" s="22" t="inlineStr">
-        <is>
-          <t>조작자가 경고 상태에서 동작을 강행했습니다.</t>
-        </is>
-      </c>
-      <c r="I134" s="22" t="inlineStr">
-        <is>
-          <t>강행 사유를 기록하십시오</t>
-        </is>
-      </c>
-      <c r="J134" s="20" t="inlineStr"/>
-      <c r="K134" s="19" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="23" t="n">
-        <v>8002</v>
-      </c>
-      <c r="B135" s="24" t="inlineStr">
-        <is>
-          <t>AUDIT_CONFIG_CHANGED</t>
-        </is>
-      </c>
-      <c r="C135" s="23" t="inlineStr">
-        <is>
-          <t>정보</t>
-        </is>
-      </c>
-      <c r="D135" s="23" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E135" s="25" t="inlineStr">
-        <is>
-          <t>조작 이력</t>
-        </is>
-      </c>
-      <c r="F135" s="25" t="inlineStr">
-        <is>
-          <t>관제</t>
-        </is>
-      </c>
-      <c r="G135" s="26" t="inlineStr">
-        <is>
-          <t>설정 변경</t>
-        </is>
-      </c>
-      <c r="H135" s="26" t="inlineStr">
-        <is>
-          <t>조작자가 설정을 변경했습니다.</t>
-        </is>
-      </c>
-      <c r="I135" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J135" s="24" t="inlineStr"/>
-      <c r="K135" s="23" t="inlineStr"/>
+      <c r="K135" s="19" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="23" t="n">
+        <v>7003</v>
+      </c>
+      <c r="B136" s="24" t="inlineStr">
+        <is>
+          <t>POWER_RETURN_TO_DOCK</t>
+        </is>
+      </c>
+      <c r="C136" s="23" t="inlineStr">
+        <is>
+          <t>정보</t>
+        </is>
+      </c>
+      <c r="D136" s="23" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E136" s="25" t="inlineStr">
+        <is>
+          <t>전원</t>
+        </is>
+      </c>
+      <c r="F136" s="25" t="inlineStr">
+        <is>
+          <t>미션 FSM</t>
+        </is>
+      </c>
+      <c r="G136" s="26" t="inlineStr">
+        <is>
+          <t>충전 스테이션 복귀</t>
+        </is>
+      </c>
+      <c r="H136" s="26" t="inlineStr">
+        <is>
+          <t>점검 완료 또는 배터리 부족으로 복귀 중입니다.</t>
+        </is>
+      </c>
+      <c r="I136" s="26" t="inlineStr">
+        <is>
+          <t>복귀 경로상 장애물이 없는지 확인하십시오</t>
+        </is>
+      </c>
+      <c r="J136" s="24" t="inlineStr">
+        <is>
+          <t>state/mission</t>
+        </is>
+      </c>
+      <c r="K136" s="23" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="27" t="n">
+        <v>7004</v>
+      </c>
+      <c r="B137" s="28" t="inlineStr">
+        <is>
+          <t>POWER_DOCKED</t>
+        </is>
+      </c>
+      <c r="C137" s="27" t="inlineStr">
+        <is>
+          <t>정상</t>
+        </is>
+      </c>
+      <c r="D137" s="27" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E137" s="29" t="inlineStr">
+        <is>
+          <t>전원</t>
+        </is>
+      </c>
+      <c r="F137" s="29" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="G137" s="30" t="inlineStr">
+        <is>
+          <t>충전 스테이션 도킹 완료</t>
+        </is>
+      </c>
+      <c r="H137" s="30" t="inlineStr">
+        <is>
+          <t>복귀와 충전 연결이 완료되었습니다.</t>
+        </is>
+      </c>
+      <c r="I137" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J137" s="28" t="inlineStr">
+        <is>
+          <t>state/mission</t>
+        </is>
+      </c>
+      <c r="K137" s="27" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="19" t="n">
+        <v>8001</v>
+      </c>
+      <c r="B138" s="20" t="inlineStr">
+        <is>
+          <t>AUDIT_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="C138" s="19" t="inlineStr">
+        <is>
+          <t>경고</t>
+        </is>
+      </c>
+      <c r="D138" s="19" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E138" s="21" t="inlineStr">
+        <is>
+          <t>조작 이력</t>
+        </is>
+      </c>
+      <c r="F138" s="21" t="inlineStr">
+        <is>
+          <t>관제</t>
+        </is>
+      </c>
+      <c r="G138" s="22" t="inlineStr">
+        <is>
+          <t>경고를 무시하고 강행</t>
+        </is>
+      </c>
+      <c r="H138" s="22" t="inlineStr">
+        <is>
+          <t>조작자가 경고 상태에서 동작을 강행했습니다.</t>
+        </is>
+      </c>
+      <c r="I138" s="22" t="inlineStr">
+        <is>
+          <t>강행 사유를 기록하십시오</t>
+        </is>
+      </c>
+      <c r="J138" s="20" t="inlineStr"/>
+      <c r="K138" s="19" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="23" t="n">
+        <v>8002</v>
+      </c>
+      <c r="B139" s="24" t="inlineStr">
+        <is>
+          <t>AUDIT_CONFIG_CHANGED</t>
+        </is>
+      </c>
+      <c r="C139" s="23" t="inlineStr">
+        <is>
+          <t>정보</t>
+        </is>
+      </c>
+      <c r="D139" s="23" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E139" s="25" t="inlineStr">
+        <is>
+          <t>조작 이력</t>
+        </is>
+      </c>
+      <c r="F139" s="25" t="inlineStr">
+        <is>
+          <t>관제</t>
+        </is>
+      </c>
+      <c r="G139" s="26" t="inlineStr">
+        <is>
+          <t>설정 변경</t>
+        </is>
+      </c>
+      <c r="H139" s="26" t="inlineStr">
+        <is>
+          <t>조작자가 설정을 변경했습니다.</t>
+        </is>
+      </c>
+      <c r="I139" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J139" s="24" t="inlineStr"/>
+      <c r="K139" s="23" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="23" t="n">
         <v>8003</v>
       </c>
-      <c r="B136" s="24" t="inlineStr">
+      <c r="B140" s="24" t="inlineStr">
         <is>
           <t>AUDIT_SIGNIN</t>
         </is>
       </c>
-      <c r="C136" s="23" t="inlineStr">
+      <c r="C140" s="23" t="inlineStr">
         <is>
           <t>정보</t>
         </is>
       </c>
-      <c r="D136" s="23" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E136" s="25" t="inlineStr">
+      <c r="D140" s="23" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E140" s="25" t="inlineStr">
         <is>
           <t>조작 이력</t>
         </is>
       </c>
-      <c r="F136" s="25" t="inlineStr">
+      <c r="F140" s="25" t="inlineStr">
         <is>
           <t>관제</t>
         </is>
       </c>
-      <c r="G136" s="26" t="inlineStr">
+      <c r="G140" s="26" t="inlineStr">
         <is>
           <t>조작자 로그인</t>
         </is>
       </c>
-      <c r="H136" s="26" t="inlineStr">
+      <c r="H140" s="26" t="inlineStr">
         <is>
           <t>관제 화면에 조작자가 로그인했습니다.</t>
         </is>
       </c>
-      <c r="I136" s="26" t="inlineStr">
+      <c r="I140" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J136" s="24" t="inlineStr"/>
-      <c r="K136" s="23" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="23" t="n">
+      <c r="J140" s="24" t="inlineStr"/>
+      <c r="K140" s="23" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="23" t="n">
         <v>8004</v>
       </c>
-      <c r="B137" s="24" t="inlineStr">
+      <c r="B141" s="24" t="inlineStr">
         <is>
           <t>AUDIT_SIGNOUT</t>
         </is>
       </c>
-      <c r="C137" s="23" t="inlineStr">
+      <c r="C141" s="23" t="inlineStr">
         <is>
           <t>정보</t>
         </is>
       </c>
-      <c r="D137" s="23" t="inlineStr">
-        <is>
-          <t>1회</t>
-        </is>
-      </c>
-      <c r="E137" s="25" t="inlineStr">
+      <c r="D141" s="23" t="inlineStr">
+        <is>
+          <t>1회</t>
+        </is>
+      </c>
+      <c r="E141" s="25" t="inlineStr">
         <is>
           <t>조작 이력</t>
         </is>
       </c>
-      <c r="F137" s="25" t="inlineStr">
+      <c r="F141" s="25" t="inlineStr">
         <is>
           <t>관제</t>
         </is>
       </c>
-      <c r="G137" s="26" t="inlineStr">
+      <c r="G141" s="26" t="inlineStr">
         <is>
           <t>조작자 로그아웃</t>
         </is>
       </c>
-      <c r="H137" s="26" t="inlineStr">
+      <c r="H141" s="26" t="inlineStr">
         <is>
           <t>관제 화면에서 조작자가 로그아웃했습니다.</t>
         </is>
       </c>
-      <c r="I137" s="26" t="inlineStr">
+      <c r="I141" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J137" s="24" t="inlineStr"/>
-      <c r="K137" s="23" t="inlineStr"/>
+      <c r="J141" s="24" t="inlineStr"/>
+      <c r="K141" s="23" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K137"/>
+  <autoFilter ref="A1:K141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>